<commit_message>
add roteamento de erros
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos\Glowi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95FC7DE3-7767-4DDA-B767-8005F2C98474}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FAC81D1-6CB4-4B46-9C90-85B78FE2E263}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="128">
   <si>
     <t>BACKLOG DO PRODUTO — Todas as Ondas até o MVP</t>
   </si>
@@ -421,6 +421,9 @@
   </si>
   <si>
     <t>#04</t>
+  </si>
+  <si>
+    <t>#05</t>
   </si>
 </sst>
 </file>
@@ -1251,8 +1254,12 @@
       <c r="F9" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="G9" s="13"/>
-      <c r="H9" s="12"/>
+      <c r="G9" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="H9" s="12" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="10" spans="1:17" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="12" t="s">

</xml_diff>

<commit_message>
transforma app em PWA
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos\Glowi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C36BAE5B-B076-42ED-A881-2D76333AB6E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{503CF489-DA57-47C7-9252-A096340E6C30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="INSTRUÇÕES" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">BACKLOG!$A$4:$H$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">BACKLOG!$A$4:$H$15</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="129">
   <si>
     <t>BACKLOG DO PRODUTO — Todas as Ondas até o MVP</t>
   </si>
@@ -144,9 +144,6 @@
     <t>T10</t>
   </si>
   <si>
-    <t>T11</t>
-  </si>
-  <si>
     <t>F05</t>
   </si>
   <si>
@@ -427,6 +424,9 @@
   </si>
   <si>
     <t>#06</t>
+  </si>
+  <si>
+    <t>Iago</t>
   </si>
 </sst>
 </file>
@@ -619,7 +619,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -709,6 +709,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1108,19 +1111,19 @@
         <v>28</v>
       </c>
       <c r="E5" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="G5" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="F5" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="G5" s="13" t="s">
-        <v>70</v>
-      </c>
       <c r="H5" s="12" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J5" s="32" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K5" s="28"/>
       <c r="L5" s="28"/>
@@ -1144,20 +1147,20 @@
         <v>17</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F6" s="13" t="s">
         <v>32</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H6" s="12" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J6" s="3"/>
       <c r="K6" s="27" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L6" s="28"/>
       <c r="M6" s="28"/>
@@ -1180,20 +1183,20 @@
         <v>19</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H7" s="12" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="27" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="L7" s="28"/>
       <c r="M7" s="28"/>
@@ -1216,20 +1219,20 @@
         <v>17</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F8" s="13" t="s">
         <v>32</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J8" s="5"/>
       <c r="K8" s="27" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="L8" s="28"/>
       <c r="M8" s="28"/>
@@ -1252,16 +1255,16 @@
         <v>19</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F9" s="13" t="s">
         <v>32</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="10" spans="1:17" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
@@ -1278,19 +1281,19 @@
         <v>17</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F10" s="13" t="s">
         <v>32</v>
       </c>
       <c r="G10" s="13" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J10" s="32" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="K10" s="28"/>
       <c r="L10" s="28"/>
@@ -1314,18 +1317,20 @@
         <v>17</v>
       </c>
       <c r="E11" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="F11" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="F11" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="G11" s="13"/>
+      <c r="G11" s="13" t="s">
+        <v>128</v>
+      </c>
       <c r="H11" s="12"/>
       <c r="J11" s="6" t="s">
         <v>9</v>
       </c>
       <c r="K11" s="27" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="L11" s="28"/>
       <c r="M11" s="28"/>
@@ -1348,18 +1353,20 @@
         <v>19</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F12" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="G12" s="13"/>
+      <c r="G12" s="13" t="s">
+        <v>128</v>
+      </c>
       <c r="H12" s="12"/>
       <c r="J12" s="6" t="s">
         <v>11</v>
       </c>
       <c r="K12" s="27" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="L12" s="28"/>
       <c r="M12" s="28"/>
@@ -1382,18 +1389,20 @@
         <v>19</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F13" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="G13" s="13"/>
+      <c r="G13" s="13" t="s">
+        <v>128</v>
+      </c>
       <c r="H13" s="12"/>
       <c r="J13" s="6" t="s">
         <v>13</v>
       </c>
       <c r="K13" s="27" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L13" s="28"/>
       <c r="M13" s="28"/>
@@ -1413,60 +1422,70 @@
         <v>25</v>
       </c>
       <c r="D14" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="E14" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="E14" s="14" t="s">
-        <v>81</v>
-      </c>
       <c r="F14" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="G14" s="13"/>
+        <v>36</v>
+      </c>
+      <c r="G14" s="13" t="s">
+        <v>128</v>
+      </c>
       <c r="H14" s="12"/>
     </row>
     <row r="15" spans="1:17" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="15" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B15" s="15" t="s">
         <v>15</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="D15" s="15"/>
-      <c r="E15" s="16"/>
+        <v>16</v>
+      </c>
+      <c r="D15" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E15" s="16" t="s">
+        <v>81</v>
+      </c>
       <c r="F15" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="G15" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="H15" s="15"/>
+    </row>
+    <row r="16" spans="1:17" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="B16" s="21" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="D16" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="E16" s="22" t="s">
+        <v>84</v>
+      </c>
+      <c r="F16" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
-    </row>
-    <row r="16" spans="1:17" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="B16" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="C16" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="D16" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="E16" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="F16" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="G16" s="15"/>
-      <c r="H16" s="15"/>
+      <c r="G16" s="35" t="s">
+        <v>69</v>
+      </c>
+      <c r="H16" s="20"/>
     </row>
     <row r="17" spans="1:10" ht="39" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="20" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B17" s="21" t="s">
         <v>30</v>
@@ -1478,7 +1497,7 @@
         <v>19</v>
       </c>
       <c r="E17" s="22" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F17" s="21" t="s">
         <v>32</v>
@@ -1488,19 +1507,19 @@
     </row>
     <row r="18" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="20" t="s">
-        <v>41</v>
+        <v>82</v>
       </c>
       <c r="B18" s="21" t="s">
         <v>30</v>
       </c>
       <c r="C18" s="21" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D18" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="E18" s="22" t="s">
-        <v>87</v>
+        <v>17</v>
+      </c>
+      <c r="E18" s="24" t="s">
+        <v>121</v>
       </c>
       <c r="F18" s="21" t="s">
         <v>32</v>
@@ -1516,60 +1535,60 @@
         <v>30</v>
       </c>
       <c r="C19" s="21" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D19" s="21" t="s">
-        <v>17</v>
-      </c>
-      <c r="E19" s="24" t="s">
-        <v>122</v>
+        <v>19</v>
+      </c>
+      <c r="E19" s="22" t="s">
+        <v>89</v>
       </c>
       <c r="F19" s="21" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G19" s="21"/>
       <c r="H19" s="20"/>
     </row>
     <row r="20" spans="1:10" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="20" t="s">
-        <v>84</v>
-      </c>
-      <c r="B20" s="21" t="s">
-        <v>30</v>
-      </c>
-      <c r="C20" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="D20" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="E20" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="F20" s="21" t="s">
-        <v>37</v>
-      </c>
-      <c r="G20" s="21"/>
-      <c r="H20" s="20"/>
+      <c r="A20" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="B20" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="C20" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="D20" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="E20" s="19" t="s">
+        <v>92</v>
+      </c>
+      <c r="F20" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G20" s="18"/>
+      <c r="H20" s="17"/>
     </row>
     <row r="21" spans="1:10" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="17" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B21" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="C21" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="C21" s="18" t="s">
-        <v>40</v>
-      </c>
       <c r="D21" s="18" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E21" s="19" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G21" s="18"/>
       <c r="H21" s="17"/>
@@ -1579,38 +1598,38 @@
         <v>88</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C22" s="18" t="s">
-        <v>40</v>
+        <v>96</v>
       </c>
       <c r="D22" s="18" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="E22" s="19" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F22" s="18" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="G22" s="18"/>
       <c r="H22" s="17"/>
     </row>
     <row r="23" spans="1:10" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="17" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D23" s="18" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="E23" s="19" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F23" s="18" t="s">
         <v>32</v>
@@ -1619,42 +1638,42 @@
       <c r="H23" s="17"/>
     </row>
     <row r="24" spans="1:10" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="17" t="s">
+      <c r="A24" s="25" t="s">
         <v>91</v>
       </c>
-      <c r="B24" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="C24" s="18" t="s">
-        <v>97</v>
-      </c>
-      <c r="D24" s="18" t="s">
-        <v>17</v>
-      </c>
-      <c r="E24" s="19" t="s">
-        <v>100</v>
-      </c>
-      <c r="F24" s="18" t="s">
+      <c r="B24" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="C24" s="25" t="s">
+        <v>96</v>
+      </c>
+      <c r="D24" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="E24" s="26" t="s">
+        <v>101</v>
+      </c>
+      <c r="F24" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="G24" s="18"/>
-      <c r="H24" s="17"/>
+      <c r="G24" s="25"/>
+      <c r="H24" s="25"/>
     </row>
     <row r="25" spans="1:10" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="25" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B25" s="25" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C25" s="25" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="D25" s="25" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E25" s="26" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F25" s="25" t="s">
         <v>32</v>
@@ -1663,133 +1682,133 @@
       <c r="H25" s="25"/>
     </row>
     <row r="26" spans="1:10" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="25" t="s">
-        <v>94</v>
-      </c>
-      <c r="B26" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="C26" s="25" t="s">
-        <v>104</v>
-      </c>
-      <c r="D26" s="25" t="s">
-        <v>17</v>
-      </c>
-      <c r="E26" s="26" t="s">
-        <v>105</v>
-      </c>
-      <c r="F26" s="25" t="s">
-        <v>32</v>
-      </c>
-      <c r="G26" s="25"/>
-      <c r="H26" s="25"/>
+      <c r="A26" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="B26" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="C26" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="D26" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="E26" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="F26" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G26" s="18"/>
+      <c r="H26" s="17"/>
     </row>
     <row r="27" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="17" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B27" s="18" t="s">
-        <v>39</v>
+        <v>109</v>
       </c>
       <c r="C27" s="18" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="D27" s="18" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E27" s="19" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="F27" s="18" t="s">
-        <v>37</v>
+        <v>76</v>
       </c>
       <c r="G27" s="18"/>
       <c r="H27" s="17"/>
     </row>
     <row r="28" spans="1:10" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="17" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B28" s="18" t="s">
+        <v>109</v>
+      </c>
+      <c r="C28" s="18" t="s">
         <v>110</v>
-      </c>
-      <c r="C28" s="18" t="s">
-        <v>111</v>
       </c>
       <c r="D28" s="18" t="s">
         <v>17</v>
       </c>
       <c r="E28" s="19" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F28" s="18" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G28" s="18"/>
       <c r="H28" s="17"/>
     </row>
     <row r="29" spans="1:10" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="17" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B29" s="18" t="s">
+        <v>109</v>
+      </c>
+      <c r="C29" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="C29" s="18" t="s">
-        <v>111</v>
-      </c>
       <c r="D29" s="18" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E29" s="19" t="s">
         <v>114</v>
       </c>
       <c r="F29" s="18" t="s">
-        <v>77</v>
+        <v>32</v>
       </c>
       <c r="G29" s="18"/>
       <c r="H29" s="17"/>
     </row>
     <row r="30" spans="1:10" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="17" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B30" s="18" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C30" s="18" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D30" s="18" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E30" s="19" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F30" s="18" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G30" s="18"/>
       <c r="H30" s="17"/>
     </row>
     <row r="31" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="17" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B31" s="18" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C31" s="18" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D31" s="18" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E31" s="19" t="s">
         <v>117</v>
       </c>
       <c r="F31" s="18" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G31" s="18"/>
       <c r="H31" s="17"/>
@@ -1799,19 +1818,19 @@
         <v>108</v>
       </c>
       <c r="B32" s="18" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C32" s="18" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D32" s="18" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E32" s="19" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F32" s="18" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="G32" s="18"/>
       <c r="H32" s="17"/>
@@ -1819,50 +1838,29 @@
     </row>
     <row r="33" spans="1:8" ht="31.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="17" t="s">
+        <v>112</v>
+      </c>
+      <c r="B33" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="B33" s="18" t="s">
-        <v>110</v>
-      </c>
       <c r="C33" s="18" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D33" s="18" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E33" s="19" t="s">
         <v>120</v>
       </c>
       <c r="F33" s="18" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G33" s="18"/>
       <c r="H33" s="17"/>
     </row>
-    <row r="34" spans="1:8" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="17" t="s">
-        <v>113</v>
-      </c>
-      <c r="B34" s="18" t="s">
-        <v>110</v>
-      </c>
-      <c r="C34" s="18" t="s">
-        <v>119</v>
-      </c>
-      <c r="D34" s="18" t="s">
-        <v>19</v>
-      </c>
-      <c r="E34" s="19" t="s">
-        <v>121</v>
-      </c>
-      <c r="F34" s="18" t="s">
-        <v>37</v>
-      </c>
-      <c r="G34" s="18"/>
-      <c r="H34" s="17"/>
-    </row>
+    <row r="34" spans="1:8" ht="31.2" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <autoFilter ref="A4:H16" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A4:H15" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="13">
     <mergeCell ref="K11:Q11"/>
     <mergeCell ref="K8:Q8"/>
@@ -1879,6 +1877,7 @@
     <mergeCell ref="D2:E2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1893,80 +1892,80 @@
   <sheetData>
     <row r="1" spans="1:2" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="34" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B1" s="28"/>
     </row>
     <row r="2" spans="1:2" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2" s="8" t="s">
         <v>51</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3" s="10" t="s">
         <v>53</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4" s="8" t="s">
         <v>55</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" s="10" t="s">
         <v>57</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B6" s="8" t="s">
         <v>59</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="B7" s="10" t="s">
         <v>61</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>63</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="B9" s="10" t="s">
         <v>65</v>
-      </c>
-      <c r="B9" s="10" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>67</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>